<commit_message>
prism hcpb A C Th232
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-04-10.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-04-10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDDB491-F090-42F4-8E34-BB21369B9C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F315056-74B9-4FD9-A47F-3DFD3BFCFF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,43 +356,43 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.67015864678428949</c:v>
+                  <c:v>0.17624938992497577</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.67399433743759052</c:v>
+                  <c:v>0.82691997712063736</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.67258163487423628</c:v>
+                  <c:v>0.53604618365050316</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.69883311557825745</c:v>
+                  <c:v>0.67249847128047058</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.73244907600666376</c:v>
+                  <c:v>0.61540498338945215</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.76691398093902452</c:v>
+                  <c:v>0.680803562830266</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.79412199858198884</c:v>
+                  <c:v>0.77246629253567023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.82771654679092965</c:v>
+                  <c:v>0.72867315835336177</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.87277793951821403</c:v>
+                  <c:v>0.8200846093262375</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.90774216971761523</c:v>
+                  <c:v>0.84652881228569787</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.96885985849430767</c:v>
+                  <c:v>0.94926751684278332</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0035052756769365</c:v>
+                  <c:v>0.91067388980847419</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0159556160581653</c:v>
+                  <c:v>0.897241060657194</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -880,43 +880,43 @@
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>1.0001629351709587</c:v>
+                  <c:v>1.0119378821291016</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0000650261216626</c:v>
+                  <c:v>1.0179707921448478</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.99996036360746876</c:v>
+                  <c:v>1.027861427431511</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.0005266084564297</c:v>
+                  <c:v>0.98075710537859517</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0018467149465879</c:v>
+                  <c:v>0.97199820729613373</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.002287048308576</c:v>
+                  <c:v>1.0175104699823445</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0038025582102672</c:v>
+                  <c:v>1.0048750533338346</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0036838050286592</c:v>
+                  <c:v>0.9979952120781076</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.002467577491776</c:v>
+                  <c:v>1.011050091074648</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.000596548769378</c:v>
+                  <c:v>1.0131574726669086</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0015290596941282</c:v>
+                  <c:v>1.0184379609619567</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0029865814925498</c:v>
+                  <c:v>0.9965086561044354</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0003513071302839</c:v>
+                  <c:v>0.97509536567142829</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2982,43 +2982,43 @@
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.67015864678428949</c:v>
+                  <c:v>0.17624938992497577</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.67399433743759052</c:v>
+                  <c:v>0.82691997712063736</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.67258163487423628</c:v>
+                  <c:v>0.53604618365050316</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.69883311557825745</c:v>
+                  <c:v>0.67249847128047058</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.73244907600666376</c:v>
+                  <c:v>0.61540498338945215</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.76691398093902452</c:v>
+                  <c:v>0.680803562830266</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.79412199858198884</c:v>
+                  <c:v>0.77246629253567023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.82771654679092965</c:v>
+                  <c:v>0.72867315835336177</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.87277793951821403</c:v>
+                  <c:v>0.8200846093262375</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.90774216971761523</c:v>
+                  <c:v>0.84652881228569787</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.96885985849430767</c:v>
+                  <c:v>0.94926751684278332</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0035052756769365</c:v>
+                  <c:v>0.91067388980847419</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0159556160581653</c:v>
+                  <c:v>0.897241060657194</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7312,24 +7312,24 @@
       </c>
       <c r="B5" s="4"/>
       <c r="D5">
-        <v>1.3891095589010301</v>
+        <v>1.3681371012949699</v>
       </c>
       <c r="E5">
-        <v>1.02494314460544E-4</v>
+        <v>1.1475260729751101E-2</v>
       </c>
       <c r="F5">
-        <v>1.38933589370449</v>
+        <v>1.38446976074668</v>
       </c>
       <c r="G5">
-        <v>1.1377551521665301E-4</v>
+        <v>1.12587768842507E-2</v>
       </c>
       <c r="H5" s="7">
         <f t="shared" ref="H5:H17" si="0">F5/D5</f>
-        <v>1.0001629351709587</v>
+        <v>1.0119378821291016</v>
       </c>
       <c r="I5">
         <f>H5*((E5/D5)^2 +(G5/F5)^2)^0.5</f>
-        <v>1.1024684824037706E-4</v>
+        <v>1.182205369797695E-2</v>
       </c>
       <c r="J5" s="3"/>
       <c r="L5">
@@ -7359,24 +7359,24 @@
       </c>
       <c r="B6" s="4"/>
       <c r="D6">
-        <v>1.38907673010083</v>
+        <v>1.36116575463441</v>
       </c>
       <c r="E6">
-        <v>1.52707495750366E-4</v>
+        <v>1.1125190871760801E-2</v>
       </c>
       <c r="F6">
-        <v>1.3891670563732801</v>
+        <v>1.3856269814856299</v>
       </c>
       <c r="G6">
-        <v>1.6878154642812701E-4</v>
+        <v>1.0321337384108399E-2</v>
       </c>
       <c r="H6" s="7">
         <f t="shared" si="0"/>
-        <v>1.0000650261216626</v>
+        <v>1.0179707921448478</v>
       </c>
       <c r="I6">
         <f t="shared" ref="I6:I16" si="2">H6*((E6/D6)^2 +(G6/F6)^2)^0.5</f>
-        <v>1.6386259048946993E-4</v>
+        <v>1.1257118632435607E-2</v>
       </c>
       <c r="J6" s="3"/>
       <c r="L6">
@@ -7406,24 +7406,24 @@
       </c>
       <c r="B7" s="4"/>
       <c r="D7">
-        <v>1.3889139640202901</v>
+        <v>1.3663565821363799</v>
       </c>
       <c r="E7">
-        <v>1.8201886596701201E-4</v>
+        <v>1.6432050614063699E-2</v>
       </c>
       <c r="F7">
-        <v>1.3888589124812201</v>
+        <v>1.40442522689514</v>
       </c>
       <c r="G7">
-        <v>1.54337152453701E-4</v>
+        <v>1.3826122129943601E-2</v>
       </c>
       <c r="H7" s="7">
         <f t="shared" si="0"/>
-        <v>0.99996036360746876</v>
+        <v>1.027861427431511</v>
       </c>
       <c r="I7">
         <f t="shared" si="2"/>
-        <v>1.7181641313147609E-4</v>
+        <v>1.5974792343773782E-2</v>
       </c>
       <c r="J7" s="3"/>
       <c r="L7">
@@ -7453,24 +7453,24 @@
       </c>
       <c r="B8" s="4"/>
       <c r="D8">
-        <v>1.38607567014507</v>
+        <v>1.39704864054061</v>
       </c>
       <c r="E8">
-        <v>3.8958612319318502E-4</v>
+        <v>1.23281362355317E-2</v>
       </c>
       <c r="F8">
-        <v>1.3868055893142199</v>
+        <v>1.3701653807697101</v>
       </c>
       <c r="G8">
-        <v>4.0944327607914799E-4</v>
+        <v>1.18088772589459E-2</v>
       </c>
       <c r="H8" s="7">
         <f t="shared" si="0"/>
-        <v>1.0005266084564297</v>
+        <v>0.98075710537859517</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>4.0785290749755253E-4</v>
+        <v>1.2097557519592871E-2</v>
       </c>
       <c r="J8" s="3"/>
       <c r="L8">
@@ -7501,24 +7501,24 @@
       <c r="B9" s="4"/>
       <c r="C9"/>
       <c r="D9">
-        <v>1.37947186689904</v>
+        <v>1.39382815633733</v>
       </c>
       <c r="E9">
-        <v>8.86091661857925E-4</v>
+        <v>1.27595827530817E-2</v>
       </c>
       <c r="F9">
-        <v>1.3820193582140401</v>
+        <v>1.35479846923876</v>
       </c>
       <c r="G9">
-        <v>1.17898543365087E-3</v>
+        <v>1.49502540503268E-2</v>
       </c>
       <c r="H9" s="7">
         <f t="shared" si="0"/>
-        <v>1.0018467149465879</v>
+        <v>0.97199820729613373</v>
       </c>
       <c r="I9">
         <f t="shared" si="2"/>
-        <v>1.0698498708561776E-3</v>
+        <v>1.3936370030626408E-2</v>
       </c>
       <c r="K9"/>
       <c r="L9">
@@ -7548,24 +7548,24 @@
       </c>
       <c r="B10" s="4"/>
       <c r="D10">
-        <v>1.37231900559378</v>
+        <v>1.36790794333796</v>
       </c>
       <c r="E10">
-        <v>9.8135892237590492E-4</v>
+        <v>1.2545386712593301E-2</v>
       </c>
       <c r="F10">
-        <v>1.3754575654543499</v>
+        <v>1.39186065431839</v>
       </c>
       <c r="G10">
-        <v>7.1929329253824501E-4</v>
+        <v>1.3451922716281201E-2</v>
       </c>
       <c r="H10" s="7">
         <f t="shared" si="0"/>
-        <v>1.002287048308576</v>
+        <v>1.0175104699823445</v>
       </c>
       <c r="I10">
         <f t="shared" si="2"/>
-        <v>8.8794780325578441E-4</v>
+        <v>1.3556883805699941E-2</v>
       </c>
       <c r="J10" s="3"/>
       <c r="L10">
@@ -7596,24 +7596,24 @@
       <c r="B11" s="4"/>
       <c r="C11"/>
       <c r="D11">
-        <v>1.3652125452841399</v>
+        <v>1.35845231954227</v>
       </c>
       <c r="E11">
-        <v>9.36891207849102E-4</v>
+        <v>1.5737099383174798E-2</v>
       </c>
       <c r="F11">
-        <v>1.37040384545697</v>
+        <v>1.3650748470515099</v>
       </c>
       <c r="G11">
-        <v>1.1043763633645899E-3</v>
+        <v>1.2589958922203499E-2</v>
       </c>
       <c r="H11" s="7">
         <f t="shared" si="0"/>
-        <v>1.0038025582102672</v>
+        <v>1.0048750533338346</v>
       </c>
       <c r="I11">
         <f t="shared" si="2"/>
-        <v>1.0625098571799413E-3</v>
+        <v>1.4879770666968438E-2</v>
       </c>
       <c r="K11"/>
       <c r="L11">
@@ -7643,24 +7643,24 @@
       </c>
       <c r="B12" s="4"/>
       <c r="D12">
-        <v>1.35996558693921</v>
+        <v>1.3545568399108701</v>
       </c>
       <c r="E12">
-        <v>8.2269713778889005E-4</v>
+        <v>1.6297468246439701E-2</v>
       </c>
       <c r="F12">
-        <v>1.3649754350071801</v>
+        <v>1.3518412407186999</v>
       </c>
       <c r="G12">
-        <v>1.0934621564654399E-3</v>
+        <v>1.40724264166723E-2</v>
       </c>
       <c r="H12" s="7">
         <f t="shared" si="0"/>
-        <v>1.0036838050286592</v>
+        <v>0.9979952120781076</v>
       </c>
       <c r="I12">
         <f t="shared" si="2"/>
-        <v>1.0075356465859516E-3</v>
+        <v>1.5877958663557092E-2</v>
       </c>
       <c r="J12" s="3"/>
       <c r="L12">
@@ -7690,24 +7690,24 @@
       </c>
       <c r="B13" s="4"/>
       <c r="D13">
-        <v>1.3471169036955299</v>
+        <v>1.34755153312925</v>
       </c>
       <c r="E13">
-        <v>3.4192473007070602E-3</v>
+        <v>1.50714507765111E-2</v>
       </c>
       <c r="F13">
-        <v>1.35044101904588</v>
+        <v>1.36244210029811</v>
       </c>
       <c r="G13">
-        <v>3.6209913911154899E-3</v>
+        <v>1.27279533228061E-2</v>
       </c>
       <c r="H13" s="7">
         <f t="shared" si="0"/>
-        <v>1.002467577491776</v>
+        <v>1.011050091074648</v>
       </c>
       <c r="I13">
         <f t="shared" si="2"/>
-        <v>3.7012678767904027E-3</v>
+        <v>1.4733684895401899E-2</v>
       </c>
       <c r="J13" s="3"/>
       <c r="L13">
@@ -7738,24 +7738,24 @@
       <c r="B14" s="4"/>
       <c r="C14"/>
       <c r="D14">
-        <v>1.3301704109246899</v>
+        <v>1.31707186586173</v>
       </c>
       <c r="E14">
-        <v>2.6701333301032298E-3</v>
+        <v>1.8033196660722998E-2</v>
       </c>
       <c r="F14">
-        <v>1.3309639224463901</v>
+        <v>1.3344012029371599</v>
       </c>
       <c r="G14">
-        <v>2.6466416072152398E-3</v>
+        <v>1.0229483755041201E-2</v>
       </c>
       <c r="H14" s="7">
         <f t="shared" si="0"/>
-        <v>1.000596548769378</v>
+        <v>1.0131574726669086</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
-        <v>2.8272285541985462E-3</v>
+        <v>1.5898337852427311E-2</v>
       </c>
       <c r="K14"/>
       <c r="L14">
@@ -7785,24 +7785,24 @@
       </c>
       <c r="B15" s="4"/>
       <c r="D15">
-        <v>1.2881810524951001</v>
+        <v>1.28457233028475</v>
       </c>
       <c r="E15">
-        <v>2.82817615567389E-3</v>
+        <v>1.0625495333578599E-2</v>
       </c>
       <c r="F15">
-        <v>1.2901507582212099</v>
+        <v>1.3082572247633499</v>
       </c>
       <c r="G15">
-        <v>3.6382982434454399E-3</v>
+        <v>1.23666556549391E-2</v>
       </c>
       <c r="H15" s="7">
         <f t="shared" si="0"/>
-        <v>1.0015290596941282</v>
+        <v>1.0184379609619567</v>
       </c>
       <c r="I15">
         <f t="shared" si="2"/>
-        <v>3.579377630249193E-3</v>
+        <v>1.2792431657530358E-2</v>
       </c>
       <c r="J15" s="3"/>
       <c r="L15">
@@ -7833,24 +7833,24 @@
       <c r="B16" s="4"/>
       <c r="C16"/>
       <c r="D16">
-        <v>1.24999214529804</v>
+        <v>1.2590558964513201</v>
       </c>
       <c r="E16">
-        <v>2.36320017159778E-3</v>
+        <v>1.6651460486491101E-2</v>
       </c>
       <c r="F16">
-        <v>1.2537253487050199</v>
+        <v>1.2546600993330701</v>
       </c>
       <c r="G16">
-        <v>3.5797440463882701E-3</v>
+        <v>1.314485012796E-2</v>
       </c>
       <c r="H16" s="7">
         <f t="shared" si="0"/>
-        <v>1.0029865814925498</v>
+        <v>0.9965086561044354</v>
       </c>
       <c r="I16">
         <f t="shared" si="2"/>
-        <v>3.4346863492251559E-3</v>
+        <v>1.6813371889030006E-2</v>
       </c>
       <c r="K16"/>
       <c r="L16">
@@ -7880,24 +7880,24 @@
       </c>
       <c r="B17" s="4"/>
       <c r="D17">
-        <v>1.2159170927577201</v>
+        <v>1.22750944273163</v>
       </c>
       <c r="E17">
-        <v>3.1109769949112399E-3</v>
+        <v>1.30680187336338E-2</v>
       </c>
       <c r="F17">
-        <v>1.2163442531022399</v>
+        <v>1.19693876892553</v>
       </c>
       <c r="G17">
-        <v>3.18424238805618E-3</v>
+        <v>1.11150087961693E-2</v>
       </c>
       <c r="H17" s="7">
         <f t="shared" si="0"/>
-        <v>1.0003513071302839</v>
+        <v>0.97509536567142829</v>
       </c>
       <c r="I17">
         <f>H17*((E17/D17)^2 +(G17/F17)^2)^0.5</f>
-        <v>3.6618101886275135E-3</v>
+        <v>1.377509712299383E-2</v>
       </c>
       <c r="J17" s="3"/>
       <c r="L17">
@@ -8012,24 +8012,24 @@
       <c r="B24" s="4"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2">
-        <v>3.4601339198647797E-5</v>
+        <v>3.3571202768168298E-5</v>
       </c>
       <c r="E24" s="2">
-        <v>1.22883732368375E-8</v>
+        <v>9.9159126214562193E-7</v>
       </c>
       <c r="F24" s="2">
-        <v>2.3188386654289999E-5</v>
+        <v>5.9169040069373203E-6</v>
       </c>
       <c r="G24" s="2">
-        <v>2.5713213345718999E-7</v>
+        <v>1.2392053149366401E-6</v>
       </c>
       <c r="H24" s="13">
         <f t="shared" ref="H24:H36" si="4">F24/D24</f>
-        <v>0.67015864678428949</v>
+        <v>0.17624938992497577</v>
       </c>
       <c r="I24">
         <f>H24*((E24/D24)^2 +(G24/F24)^2)^0.5</f>
-        <v>7.4350871718769813E-3</v>
+        <v>3.7278036250492967E-2</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="2"/>
@@ -8059,25 +8059,25 @@
         <v>0.5</v>
       </c>
       <c r="B25" s="4"/>
-      <c r="D25">
-        <v>1.7267075850167999E-4</v>
+      <c r="D25" s="2">
+        <v>1.67215009194801E-4</v>
       </c>
       <c r="E25" s="2">
-        <v>7.3730405114227898E-8</v>
-      </c>
-      <c r="F25">
-        <v>1.16379113471186E-4</v>
+        <v>6.3599673665714699E-6</v>
+      </c>
+      <c r="F25" s="2">
+        <v>1.3827343157759201E-4</v>
       </c>
       <c r="G25" s="2">
-        <v>4.9685826902563597E-7</v>
+        <v>3.1803156900076102E-5</v>
       </c>
       <c r="H25" s="13">
         <f t="shared" si="4"/>
-        <v>0.67399433743759052</v>
+        <v>0.82691997712063736</v>
       </c>
       <c r="I25">
         <f t="shared" ref="I25:I35" si="6">H25*((E25/D25)^2 +(G25/F25)^2)^0.5</f>
-        <v>2.8918456475792078E-3</v>
+        <v>0.19277618205248812</v>
       </c>
       <c r="J25" s="3"/>
       <c r="L25">
@@ -8106,25 +8106,25 @@
         <v>1</v>
       </c>
       <c r="B26" s="4"/>
-      <c r="D26">
-        <v>3.4444202449192702E-4</v>
+      <c r="D26" s="2">
+        <v>3.4693843594753001E-4</v>
       </c>
       <c r="E26" s="2">
-        <v>1.02701859340892E-7</v>
-      </c>
-      <c r="F26">
-        <v>2.31665379952172E-4</v>
+        <v>8.7539530299504897E-6</v>
+      </c>
+      <c r="F26" s="2">
+        <v>1.85975024551348E-4</v>
       </c>
       <c r="G26" s="2">
-        <v>6.9232886194979901E-7</v>
+        <v>3.83737519740559E-5</v>
       </c>
       <c r="H26" s="13">
         <f t="shared" si="4"/>
-        <v>0.67258163487423628</v>
+        <v>0.53604618365050316</v>
       </c>
       <c r="I26">
         <f t="shared" si="6"/>
-        <v>2.0199806972425911E-3</v>
+        <v>0.11143071864844456</v>
       </c>
       <c r="J26" s="3"/>
       <c r="L26">
@@ -8153,25 +8153,25 @@
         <v>10</v>
       </c>
       <c r="B27" s="4"/>
-      <c r="D27">
-        <v>3.33054467027722E-3</v>
+      <c r="D27" s="2">
+        <v>3.2447100360010698E-3</v>
       </c>
       <c r="E27" s="2">
-        <v>3.1023196230951202E-6</v>
-      </c>
-      <c r="F27">
-        <v>2.3274949085023899E-3</v>
+        <v>9.6341313668401696E-5</v>
+      </c>
+      <c r="F27" s="2">
+        <v>2.1820625389591202E-3</v>
       </c>
       <c r="G27" s="2">
-        <v>7.3576810457546899E-6</v>
+        <v>2.65966276223607E-4</v>
       </c>
       <c r="H27" s="13">
         <f t="shared" si="4"/>
-        <v>0.69883311557825745</v>
+        <v>0.67249847128047058</v>
       </c>
       <c r="I27">
         <f t="shared" si="6"/>
-        <v>2.3030599218682355E-3</v>
+        <v>8.4366214657354846E-2</v>
       </c>
       <c r="J27" s="3"/>
       <c r="L27">
@@ -8200,25 +8200,25 @@
         <v>25</v>
       </c>
       <c r="B28" s="4"/>
-      <c r="D28">
-        <v>7.9007108136224906E-3</v>
+      <c r="D28" s="2">
+        <v>8.1578715103711296E-3</v>
       </c>
       <c r="E28" s="2">
-        <v>2.1579374269995798E-5</v>
-      </c>
-      <c r="F28">
-        <v>5.7868683352336496E-3</v>
+        <v>2.7906538103478998E-4</v>
+      </c>
+      <c r="F28" s="2">
+        <v>5.02039478133323E-3</v>
       </c>
       <c r="G28" s="2">
-        <v>2.2153397083295701E-5</v>
+        <v>3.0805666033860603E-4</v>
       </c>
       <c r="H28" s="13">
         <f t="shared" si="4"/>
-        <v>0.73244907600666376</v>
+        <v>0.61540498338945215</v>
       </c>
       <c r="I28">
         <f t="shared" si="6"/>
-        <v>3.444486925796071E-3</v>
+        <v>4.323355798647284E-2</v>
       </c>
       <c r="J28" s="3"/>
       <c r="L28">
@@ -8247,25 +8247,25 @@
         <v>50</v>
       </c>
       <c r="B29" s="4"/>
-      <c r="D29">
-        <v>1.48099690035684E-2</v>
+      <c r="D29" s="2">
+        <v>1.49266627971049E-2</v>
       </c>
       <c r="E29" s="2">
-        <v>3.5619384608241799E-5</v>
-      </c>
-      <c r="F29">
-        <v>1.1357972286110201E-2</v>
+        <v>4.9518780486686295E-4</v>
+      </c>
+      <c r="F29" s="2">
+        <v>1.0162125213435E-2</v>
       </c>
       <c r="G29" s="2">
-        <v>3.9960656049596501E-5</v>
+        <v>5.80825745840268E-4</v>
       </c>
       <c r="H29" s="13">
         <f t="shared" si="4"/>
-        <v>0.76691398093902452</v>
+        <v>0.680803562830266</v>
       </c>
       <c r="I29">
         <f t="shared" si="6"/>
-        <v>3.2684265997479276E-3</v>
+        <v>4.4991600045113711E-2</v>
       </c>
       <c r="J29" s="3"/>
       <c r="L29">
@@ -8294,25 +8294,25 @@
         <v>75</v>
       </c>
       <c r="B30" s="4"/>
-      <c r="D30">
-        <v>2.1060130702738999E-2</v>
+      <c r="D30" s="2">
+        <v>2.1432078952745001E-2</v>
       </c>
       <c r="E30" s="2">
-        <v>3.0830038687911403E-5</v>
-      </c>
-      <c r="F30">
-        <v>1.6724313084056999E-2</v>
+        <v>5.7708761237754895E-4</v>
+      </c>
+      <c r="F30" s="2">
+        <v>1.65555585699587E-2</v>
       </c>
       <c r="G30" s="2">
-        <v>4.6773312275541899E-5</v>
+        <v>8.4894750486791501E-4</v>
       </c>
       <c r="H30" s="13">
         <f t="shared" si="4"/>
-        <v>0.79412199858198884</v>
+        <v>0.77246629253567023</v>
       </c>
       <c r="I30">
         <f t="shared" si="6"/>
-        <v>2.506797039006772E-3</v>
+        <v>4.473995917320344E-2</v>
       </c>
       <c r="J30" s="3"/>
       <c r="L30">
@@ -8341,25 +8341,25 @@
         <v>100</v>
       </c>
       <c r="B31" s="4"/>
-      <c r="D31">
-        <v>2.67600755292417E-2</v>
+      <c r="D31" s="2">
+        <v>2.7913216674849899E-2</v>
       </c>
       <c r="E31" s="2">
-        <v>6.1301138330409899E-5</v>
-      </c>
-      <c r="F31">
-        <v>2.2149757308928399E-2</v>
+        <v>6.6669793207153904E-4</v>
+      </c>
+      <c r="F31" s="2">
+        <v>2.0339611754264599E-2</v>
       </c>
       <c r="G31" s="2">
-        <v>5.1020148947823797E-5</v>
+        <v>7.3633525085197403E-4</v>
       </c>
       <c r="H31" s="13">
         <f t="shared" si="4"/>
-        <v>0.82771654679092965</v>
+        <v>0.72867315835336177</v>
       </c>
       <c r="I31">
         <f t="shared" si="6"/>
-        <v>2.6889139523652702E-3</v>
+        <v>3.1603458194463079E-2</v>
       </c>
       <c r="J31" s="3"/>
       <c r="L31">
@@ -8388,25 +8388,25 @@
         <v>150</v>
       </c>
       <c r="B32" s="4"/>
-      <c r="D32">
-        <v>3.6782709718709998E-2</v>
-      </c>
-      <c r="E32">
-        <v>1.97489580151579E-4</v>
-      </c>
-      <c r="F32">
-        <v>3.2103137598192298E-2</v>
-      </c>
-      <c r="G32">
-        <v>2.08831333646651E-4</v>
+      <c r="D32" s="2">
+        <v>3.6427579453755798E-2</v>
+      </c>
+      <c r="E32" s="2">
+        <v>1.0472429250006801E-3</v>
+      </c>
+      <c r="F32" s="2">
+        <v>2.9873697265033802E-2</v>
+      </c>
+      <c r="G32" s="2">
+        <v>8.5514874767622401E-4</v>
       </c>
       <c r="H32" s="13">
         <f t="shared" si="4"/>
-        <v>0.87277793951821403</v>
+        <v>0.8200846093262375</v>
       </c>
       <c r="I32">
         <f t="shared" si="6"/>
-        <v>7.3615233968889766E-3</v>
+        <v>3.327059479181485E-2</v>
       </c>
       <c r="J32" s="3"/>
       <c r="L32">
@@ -8435,25 +8435,25 @@
         <v>250</v>
       </c>
       <c r="B33" s="4"/>
-      <c r="D33">
-        <v>5.6309750104400702E-2</v>
-      </c>
-      <c r="E33">
-        <v>2.51687827781958E-4</v>
-      </c>
-      <c r="F33">
-        <v>5.1114734736025402E-2</v>
-      </c>
-      <c r="G33">
-        <v>2.8833834514146198E-4</v>
+      <c r="D33" s="2">
+        <v>5.53819360171761E-2</v>
+      </c>
+      <c r="E33" s="2">
+        <v>1.4584466490748199E-3</v>
+      </c>
+      <c r="F33" s="2">
+        <v>4.6882404518702597E-2</v>
+      </c>
+      <c r="G33" s="2">
+        <v>9.0297433456597396E-4</v>
       </c>
       <c r="H33" s="13">
         <f t="shared" si="4"/>
-        <v>0.90774216971761523</v>
+        <v>0.84652881228569787</v>
       </c>
       <c r="I33">
         <f t="shared" si="6"/>
-        <v>6.5331679556135417E-3</v>
+        <v>2.7618912628068853E-2</v>
       </c>
       <c r="J33" s="3"/>
       <c r="L33">
@@ -8482,25 +8482,25 @@
         <v>500</v>
       </c>
       <c r="B34" s="4"/>
-      <c r="D34">
-        <v>9.4384365104793602E-2</v>
-      </c>
-      <c r="E34">
-        <v>3.7802904257795602E-4</v>
-      </c>
-      <c r="F34">
-        <v>9.1445222619505398E-2</v>
-      </c>
-      <c r="G34">
-        <v>4.4906828447954003E-4</v>
+      <c r="D34" s="2">
+        <v>9.4183377970993604E-2</v>
+      </c>
+      <c r="E34" s="2">
+        <v>1.5799693791771401E-3</v>
+      </c>
+      <c r="F34" s="2">
+        <v>8.9405221334390397E-2</v>
+      </c>
+      <c r="G34" s="2">
+        <v>1.70807591224624E-3</v>
       </c>
       <c r="H34" s="13">
         <f t="shared" si="4"/>
-        <v>0.96885985849430767</v>
+        <v>0.94926751684278332</v>
       </c>
       <c r="I34">
         <f t="shared" si="6"/>
-        <v>6.1396636178584303E-3</v>
+        <v>2.4134786583998237E-2</v>
       </c>
       <c r="J34" s="3"/>
       <c r="L34">
@@ -8529,25 +8529,25 @@
         <v>750</v>
       </c>
       <c r="B35" s="4"/>
-      <c r="D35">
-        <v>0.12681392305883499</v>
-      </c>
-      <c r="E35">
-        <v>3.7117560576619898E-4</v>
-      </c>
-      <c r="F35">
-        <v>0.12725844081883</v>
-      </c>
-      <c r="G35">
-        <v>3.9277512684765298E-4</v>
+      <c r="D35" s="2">
+        <v>0.12938440937586501</v>
+      </c>
+      <c r="E35" s="2">
+        <v>2.1442760752734399E-3</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0.117827003366891</v>
+      </c>
+      <c r="G35" s="2">
+        <v>2.1418785805969601E-3</v>
       </c>
       <c r="H35" s="13">
         <f t="shared" si="4"/>
-        <v>1.0035052756769365</v>
+        <v>0.91067388980847419</v>
       </c>
       <c r="I35">
         <f t="shared" si="6"/>
-        <v>4.2684987159538603E-3</v>
+        <v>2.2401595997311816E-2</v>
       </c>
       <c r="J35" s="3"/>
       <c r="L35">
@@ -8576,25 +8576,25 @@
         <v>999.99</v>
       </c>
       <c r="B36" s="4"/>
-      <c r="D36">
-        <v>0.15510900896549801</v>
-      </c>
-      <c r="E36">
-        <v>5.7851797067085496E-4</v>
-      </c>
-      <c r="F36">
-        <v>0.157583868759714</v>
-      </c>
-      <c r="G36">
-        <v>5.8700051779191705E-4</v>
+      <c r="D36" s="2">
+        <v>0.15752496538125499</v>
+      </c>
+      <c r="E36" s="2">
+        <v>2.4554689207597698E-3</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0.14133786701866499</v>
+      </c>
+      <c r="G36" s="2">
+        <v>1.8390528502879599E-3</v>
       </c>
       <c r="H36" s="13">
         <f t="shared" si="4"/>
-        <v>1.0159556160581653</v>
+        <v>0.897241060657194</v>
       </c>
       <c r="I36">
         <f>H36*((E36/D36)^2 +(G36/F36)^2)^0.5</f>
-        <v>5.3554157048239367E-3</v>
+        <v>1.8218310636367537E-2</v>
       </c>
       <c r="J36" s="3"/>
       <c r="L36">
@@ -8715,24 +8715,24 @@
       <c r="B42" s="4"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2">
-        <v>3.1823783667320202E-6</v>
+        <v>3.2508308570749199E-6</v>
       </c>
       <c r="E42" s="2">
-        <v>4.1159886287402301E-10</v>
+        <v>2.9879791871820602E-8</v>
       </c>
       <c r="F42" s="2">
-        <v>3.4389546303583601E-6</v>
+        <v>2.4077020934709801E-6</v>
       </c>
       <c r="G42" s="2">
-        <v>7.2754924795352899E-9</v>
+        <v>4.5116812236236001E-7</v>
       </c>
       <c r="H42" s="13">
         <f t="shared" ref="H42:H54" si="8">F42/D42</f>
-        <v>1.0806240597625159</v>
+        <v>0.74064206946694777</v>
       </c>
       <c r="I42">
         <f>H42*((E42/D42)^2 +(G42/F42)^2)^0.5</f>
-        <v>2.2904490835581361E-3</v>
+        <v>0.13895233886852032</v>
       </c>
       <c r="J42" s="3"/>
       <c r="K42" s="2"/>
@@ -8763,24 +8763,24 @@
       </c>
       <c r="B43" s="4"/>
       <c r="D43" s="2">
-        <v>1.6000871976086401E-5</v>
+        <v>1.6123275821852999E-5</v>
       </c>
       <c r="E43" s="2">
-        <v>1.8077035460066801E-9</v>
+        <v>2.0263996088365101E-7</v>
       </c>
       <c r="F43" s="2">
-        <v>1.7406241259005801E-5</v>
+        <v>1.5829821996247301E-5</v>
       </c>
       <c r="G43" s="2">
-        <v>1.6560027342357799E-8</v>
+        <v>1.9692674060295302E-6</v>
       </c>
       <c r="H43" s="13">
         <f t="shared" si="8"/>
-        <v>1.0878307935354867</v>
+        <v>0.98179936702391701</v>
       </c>
       <c r="I43">
         <f t="shared" ref="I43:I53" si="10">H43*((E43/D43)^2 +(G43/F43)^2)^0.5</f>
-        <v>1.0422167294252094E-3</v>
+        <v>0.12275990292260608</v>
       </c>
       <c r="J43" s="3"/>
       <c r="L43" s="2">
@@ -8810,24 +8810,24 @@
       </c>
       <c r="B44" s="4"/>
       <c r="D44" s="2">
-        <v>3.2035093398018297E-5</v>
+        <v>3.1996604066933298E-5</v>
       </c>
       <c r="E44" s="2">
-        <v>3.6301326712904198E-9</v>
+        <v>4.1792496489736701E-7</v>
       </c>
       <c r="F44" s="2">
-        <v>3.4905945803773603E-5</v>
+        <v>3.2983010764906299E-5</v>
       </c>
       <c r="G44" s="2">
-        <v>3.0128552778278198E-8</v>
+        <v>2.2398843673895399E-6</v>
       </c>
       <c r="H44" s="13">
         <f t="shared" si="8"/>
-        <v>1.0896158587735816</v>
+        <v>1.030828480919711</v>
       </c>
       <c r="I44">
         <f t="shared" si="10"/>
-        <v>9.4855633081543855E-4</v>
+        <v>7.1286878880722632E-2</v>
       </c>
       <c r="J44" s="3"/>
       <c r="L44" s="2">
@@ -8857,24 +8857,24 @@
       </c>
       <c r="B45" s="4"/>
       <c r="D45">
-        <v>3.2041283539142699E-4</v>
+        <v>3.17520187164021E-4</v>
       </c>
       <c r="E45" s="2">
-        <v>1.03089800141475E-7</v>
+        <v>3.5903642084798401E-6</v>
       </c>
       <c r="F45">
-        <v>3.5175355668395599E-4</v>
+        <v>3.2190498140927299E-4</v>
       </c>
       <c r="G45" s="2">
-        <v>3.24163031926656E-7</v>
+        <v>1.0083144680763101E-5</v>
       </c>
       <c r="H45" s="13">
         <f t="shared" si="8"/>
-        <v>1.0978135637239441</v>
+        <v>1.0138094975453857</v>
       </c>
       <c r="I45">
         <f t="shared" si="10"/>
-        <v>1.0715892980094322E-3</v>
+        <v>3.3761722320914872E-2</v>
       </c>
       <c r="J45" s="3"/>
       <c r="L45" s="2">
@@ -8904,24 +8904,24 @@
       </c>
       <c r="B46" s="4"/>
       <c r="D46">
-        <v>7.9832852090792796E-4</v>
+        <v>8.1568502250048002E-4</v>
       </c>
       <c r="E46" s="2">
-        <v>6.4380828459592396E-7</v>
+        <v>5.3855794471320103E-6</v>
       </c>
       <c r="F46">
-        <v>8.7467769000268295E-4</v>
+        <v>8.0308685347477604E-4</v>
       </c>
       <c r="G46" s="2">
-        <v>1.03125836480735E-6</v>
+        <v>1.5815547986996E-5</v>
       </c>
       <c r="H46" s="13">
         <f t="shared" si="8"/>
-        <v>1.0956362789192651</v>
+        <v>0.98455510561284509</v>
       </c>
       <c r="I46">
         <f t="shared" si="10"/>
-        <v>1.5650469392181556E-3</v>
+        <v>2.044997390903704E-2</v>
       </c>
       <c r="J46" s="3"/>
       <c r="L46">
@@ -8951,24 +8951,24 @@
       </c>
       <c r="B47" s="4"/>
       <c r="D47">
-        <v>1.5863990621956901E-3</v>
+        <v>1.60165101199415E-3</v>
       </c>
       <c r="E47" s="2">
-        <v>6.9872049483164404E-7</v>
+        <v>1.68217601711865E-5</v>
       </c>
       <c r="F47">
-        <v>1.7451813935783799E-3</v>
+        <v>1.64322981589001E-3</v>
       </c>
       <c r="G47" s="2">
-        <v>2.15270592824618E-6</v>
+        <v>2.5755780859259001E-5</v>
       </c>
       <c r="H47" s="13">
         <f t="shared" si="8"/>
-        <v>1.1000897789002244</v>
+        <v>1.025959964801628</v>
       </c>
       <c r="I47">
         <f t="shared" si="10"/>
-        <v>1.4408859671880526E-3</v>
+        <v>1.9357187123934069E-2</v>
       </c>
       <c r="J47" s="3"/>
       <c r="L47">
@@ -8998,24 +8998,24 @@
       </c>
       <c r="B48" s="4"/>
       <c r="D48">
-        <v>2.3694633374357899E-3</v>
+        <v>2.3979320506641501E-3</v>
       </c>
       <c r="E48" s="2">
-        <v>2.0409182758839298E-6</v>
+        <v>3.1169443646373198E-5</v>
       </c>
       <c r="F48">
-        <v>2.6035551899146001E-3</v>
+        <v>2.3274282513085498E-3</v>
       </c>
       <c r="G48" s="2">
-        <v>1.69836561383817E-6</v>
+        <v>3.8598219967931103E-5</v>
       </c>
       <c r="H48" s="13">
         <f t="shared" si="8"/>
-        <v>1.098795304734338</v>
+        <v>0.97059808290394511</v>
       </c>
       <c r="I48">
         <f t="shared" si="10"/>
-        <v>1.1872271872232696E-3</v>
+        <v>2.0451571874940244E-2</v>
       </c>
       <c r="J48" s="3"/>
       <c r="L48">
@@ -9045,24 +9045,24 @@
       </c>
       <c r="B49" s="4"/>
       <c r="D49">
-        <v>3.1410862514606899E-3</v>
+        <v>3.1150452266862499E-3</v>
       </c>
       <c r="E49" s="2">
-        <v>3.27513526933276E-6</v>
+        <v>3.0375204510835499E-5</v>
       </c>
       <c r="F49">
-        <v>3.4466944423003402E-3</v>
+        <v>3.1491175964614999E-3</v>
       </c>
       <c r="G49" s="2">
-        <v>3.2445791725811299E-6</v>
+        <v>3.7025405401571998E-5</v>
       </c>
       <c r="H49" s="13">
         <f t="shared" si="8"/>
-        <v>1.0972937915020748</v>
+        <v>1.0109380016326426</v>
       </c>
       <c r="I49">
         <f t="shared" si="10"/>
-        <v>1.541426865977242E-3</v>
+        <v>1.5441915923900233E-2</v>
       </c>
       <c r="J49" s="3"/>
       <c r="L49">
@@ -9092,24 +9092,24 @@
       </c>
       <c r="B50" s="4"/>
       <c r="D50">
-        <v>4.6445716846820698E-3</v>
+        <v>4.6543407829659003E-3</v>
       </c>
       <c r="E50" s="2">
-        <v>9.6466217564299792E-6</v>
+        <v>4.7462851945895098E-5</v>
       </c>
       <c r="F50">
-        <v>5.1102808521361299E-3</v>
+        <v>4.6288384862751501E-3</v>
       </c>
       <c r="G50" s="2">
-        <v>1.2123213047497999E-5</v>
+        <v>5.6491200849806098E-5</v>
       </c>
       <c r="H50" s="13">
         <f t="shared" si="8"/>
-        <v>1.1002695617746587</v>
+        <v>0.99452075000952134</v>
       </c>
       <c r="I50">
         <f t="shared" si="10"/>
-        <v>3.4691982513368859E-3</v>
+        <v>1.581669692140476E-2</v>
       </c>
       <c r="J50" s="3"/>
       <c r="L50">
@@ -9139,24 +9139,24 @@
       </c>
       <c r="B51" s="4"/>
       <c r="D51">
-        <v>7.5610462202649401E-3</v>
+        <v>7.6150959878939798E-3</v>
       </c>
       <c r="E51" s="2">
-        <v>1.57081565413314E-5</v>
+        <v>7.5030193636514299E-5</v>
       </c>
       <c r="F51">
-        <v>8.3558566219651704E-3</v>
+        <v>7.66287134998351E-3</v>
       </c>
       <c r="G51" s="2">
-        <v>2.3966742759134201E-5</v>
+        <v>7.5060793105698198E-5</v>
       </c>
       <c r="H51" s="13">
         <f t="shared" si="8"/>
-        <v>1.1051191036989032</v>
+        <v>1.0062737701751205</v>
       </c>
       <c r="I51">
         <f t="shared" si="10"/>
-        <v>3.9138927052399545E-3</v>
+        <v>1.398060647072992E-2</v>
       </c>
       <c r="J51" s="3"/>
       <c r="L51">
@@ -9186,24 +9186,24 @@
       </c>
       <c r="B52" s="4"/>
       <c r="D52">
-        <v>1.4415070472640399E-2</v>
-      </c>
-      <c r="E52" s="2">
-        <v>3.9280138415606102E-5</v>
+        <v>1.4555744618778E-2</v>
+      </c>
+      <c r="E52">
+        <v>1.2950150523133701E-4</v>
       </c>
       <c r="F52">
-        <v>1.57632575158239E-2</v>
-      </c>
-      <c r="G52" s="2">
-        <v>4.6556836615973601E-5</v>
+        <v>1.43182113525849E-2</v>
+      </c>
+      <c r="G52">
+        <v>1.4705046376382701E-4</v>
       </c>
       <c r="H52" s="13">
         <f t="shared" si="8"/>
-        <v>1.0935262193648196</v>
+        <v>0.9836811326102366</v>
       </c>
       <c r="I52">
         <f t="shared" si="10"/>
-        <v>4.3943507224962841E-3</v>
+        <v>1.3366190039228829E-2</v>
       </c>
       <c r="J52" s="3"/>
       <c r="L52">
@@ -9233,24 +9233,24 @@
       </c>
       <c r="B53" s="4"/>
       <c r="D53">
-        <v>2.0534104630709499E-2</v>
-      </c>
-      <c r="E53" s="2">
-        <v>5.1678598638391099E-5</v>
+        <v>2.0743350143341999E-2</v>
+      </c>
+      <c r="E53">
+        <v>2.4538469022951099E-4</v>
       </c>
       <c r="F53">
-        <v>2.23393057358535E-2</v>
-      </c>
-      <c r="G53" s="2">
-        <v>5.7826696670158199E-5</v>
+        <v>2.0707732271304301E-2</v>
+      </c>
+      <c r="G53">
+        <v>2.6747352499092303E-4</v>
       </c>
       <c r="H53" s="13">
         <f t="shared" si="8"/>
-        <v>1.0879123359702889</v>
+        <v>0.99828292576697741</v>
       </c>
       <c r="I53">
         <f t="shared" si="10"/>
-        <v>3.927730995428016E-3</v>
+        <v>1.7484977915483216E-2</v>
       </c>
       <c r="J53" s="3"/>
       <c r="L53">
@@ -9280,24 +9280,24 @@
       </c>
       <c r="B54" s="4"/>
       <c r="D54">
-        <v>2.6037643908025699E-2</v>
-      </c>
-      <c r="E54" s="2">
-        <v>7.16762407558917E-5</v>
+        <v>2.61827077319201E-2</v>
+      </c>
+      <c r="E54">
+        <v>3.1898400948727698E-4</v>
       </c>
       <c r="F54">
-        <v>2.8423944908042901E-2</v>
-      </c>
-      <c r="G54" s="2">
-        <v>6.8045831633092906E-5</v>
+        <v>2.5981087494686798E-2</v>
+      </c>
+      <c r="G54">
+        <v>4.3258976581349399E-4</v>
       </c>
       <c r="H54" s="13">
         <f t="shared" si="8"/>
-        <v>1.0916481156454276</v>
+        <v>0.99229948868170348</v>
       </c>
       <c r="I54">
         <f>H54*((E54/D54)^2 +(G54/F54)^2)^0.5</f>
-        <v>3.9824844315028184E-3</v>
+        <v>2.047251252301235E-2</v>
       </c>
       <c r="J54" s="3"/>
       <c r="L54">

</xml_diff>